<commit_message>
refactor(input): share fuel semantics and split Appendix B consumption units
</commit_message>
<xml_diff>
--- a/resources/excel_templates/gb_t_32151_34_2024_appendix_b_v2.xlsx
+++ b/resources/excel_templates/gb_t_32151_34_2024_appendix_b_v2.xlsx
@@ -1930,11 +1930,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="20" customWidth="1" style="42" min="1" max="1"/>
-    <col width="17" customWidth="1" style="42" min="2" max="2"/>
+    <col width="14" customWidth="1" style="42" min="2" max="2"/>
+    <col width="15" customWidth="1" style="42" min="3" max="3"/>
     <col width="16" customWidth="1" style="42" min="3" max="3"/>
     <col width="17" customWidth="1" style="42" min="4" max="4"/>
     <col width="15" customWidth="1" style="42" min="5" max="5"/>
@@ -1943,8 +1944,8 @@
     <col width="14" customWidth="1" style="42" min="8" max="8"/>
     <col width="17" customWidth="1" style="42" min="9" max="9"/>
     <col width="20" customWidth="1" style="42" min="10" max="10"/>
-    <col width="22" customWidth="1" style="42" min="11" max="11"/>
     <col width="22" customWidth="1" style="42" min="12" max="12"/>
+    <col width="22" customWidth="1" style="42" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="42">
@@ -1954,7 +1955,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18.45" customHeight="1" s="42">
+    <row r="2" ht="32" customHeight="1" s="42">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>燃料品种</t>
@@ -1966,89 +1967,99 @@
 t或 10⁴m³</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="43" t="n"/>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>含碳量</t>
         </is>
       </c>
-      <c r="D2" s="43" t="n"/>
-      <c r="E2" s="16" t="inlineStr">
+      <c r="E2" s="43" t="n"/>
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>低位发热量ᵃ</t>
         </is>
       </c>
-      <c r="F2" s="43" t="n"/>
-      <c r="G2" s="16" t="inlineStr">
+      <c r="G2" s="43" t="n"/>
+      <c r="H2" s="16" t="inlineStr">
         <is>
           <t>单位热值
 含碳量ᵇ
 tC/GJ</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>碳氧化率</t>
         </is>
       </c>
-      <c r="I2" s="43" t="n"/>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="J2" s="43" t="n"/>
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>排放量
 （tCO₂）</t>
         </is>
       </c>
-      <c r="K2" s="16" t="inlineStr">
+      <c r="L2" s="16" t="inlineStr">
         <is>
           <t>自定义单位热值含碳量
 （tC/GJ）</t>
         </is>
       </c>
-      <c r="L2" s="16" t="inlineStr">
+      <c r="M2" s="16" t="inlineStr">
         <is>
           <t>名称类型</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="36.1" customHeight="1" s="42">
+    <row r="3" ht="45" customHeight="1" s="42">
       <c r="A3" s="44" t="n"/>
-      <c r="B3" s="44" t="n"/>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>数据</t>
+        </is>
+      </c>
       <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>单位</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>数值
 tC/t或 tC/10⁴m³</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>数值
 GJ/t或 GJ/10⁴m³</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
       </c>
-      <c r="G3" s="44" t="n"/>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="44" t="n"/>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>数值
 %</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
       </c>
-      <c r="J3" s="44" t="n"/>
       <c r="K3" s="44" t="n"/>
       <c r="L3" s="44" t="n"/>
+      <c r="M3" s="44" t="n"/>
     </row>
     <row r="4" ht="18.05" customHeight="1" s="42">
       <c r="A4" s="46" t="inlineStr">
@@ -2058,27 +2069,28 @@
       </c>
       <c r="B4" s="47" t="n"/>
       <c r="C4" s="47" t="n"/>
-      <c r="D4" s="46" t="inlineStr">
+      <c r="D4" s="47" t="n"/>
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E4" s="47" t="n"/>
-      <c r="F4" s="46" t="inlineStr">
+      <c r="F4" s="47" t="n"/>
+      <c r="G4" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G4" s="48" t="n"/>
-      <c r="H4" s="47" t="n"/>
-      <c r="I4" s="46" t="inlineStr">
+      <c r="H4" s="48" t="n"/>
+      <c r="I4" s="47" t="n"/>
+      <c r="J4" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J4" s="49" t="str"/>
-      <c r="K4" s="46" t="n"/>
-      <c r="L4" s="46" t="inlineStr">
+      <c r="K4" s="49" t="str"/>
+      <c r="L4" s="46" t="n"/>
+      <c r="M4" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2092,27 +2104,28 @@
       </c>
       <c r="B5" s="47" t="n"/>
       <c r="C5" s="47" t="n"/>
-      <c r="D5" s="46" t="inlineStr">
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E5" s="47" t="n"/>
-      <c r="F5" s="46" t="inlineStr">
+      <c r="F5" s="47" t="n"/>
+      <c r="G5" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G5" s="48" t="n"/>
-      <c r="H5" s="47" t="n"/>
-      <c r="I5" s="46" t="inlineStr">
+      <c r="H5" s="48" t="n"/>
+      <c r="I5" s="47" t="n"/>
+      <c r="J5" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J5" s="49" t="str"/>
-      <c r="K5" s="46" t="n"/>
-      <c r="L5" s="46" t="inlineStr">
+      <c r="K5" s="49" t="str"/>
+      <c r="L5" s="46" t="n"/>
+      <c r="M5" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2126,27 +2139,28 @@
       </c>
       <c r="B6" s="47" t="n"/>
       <c r="C6" s="47" t="n"/>
-      <c r="D6" s="46" t="inlineStr">
+      <c r="D6" s="47" t="n"/>
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E6" s="47" t="n"/>
-      <c r="F6" s="46" t="inlineStr">
+      <c r="F6" s="47" t="n"/>
+      <c r="G6" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G6" s="48" t="n"/>
-      <c r="H6" s="47" t="n"/>
-      <c r="I6" s="46" t="inlineStr">
+      <c r="H6" s="48" t="n"/>
+      <c r="I6" s="47" t="n"/>
+      <c r="J6" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J6" s="49" t="str"/>
-      <c r="K6" s="46" t="n"/>
-      <c r="L6" s="46" t="inlineStr">
+      <c r="K6" s="49" t="str"/>
+      <c r="L6" s="46" t="n"/>
+      <c r="M6" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2160,27 +2174,28 @@
       </c>
       <c r="B7" s="47" t="n"/>
       <c r="C7" s="47" t="n"/>
-      <c r="D7" s="46" t="inlineStr">
+      <c r="D7" s="47" t="n"/>
+      <c r="E7" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E7" s="47" t="n"/>
-      <c r="F7" s="46" t="inlineStr">
+      <c r="F7" s="47" t="n"/>
+      <c r="G7" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G7" s="48" t="n"/>
-      <c r="H7" s="47" t="n"/>
-      <c r="I7" s="46" t="inlineStr">
+      <c r="H7" s="48" t="n"/>
+      <c r="I7" s="47" t="n"/>
+      <c r="J7" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J7" s="49" t="str"/>
-      <c r="K7" s="46" t="n"/>
-      <c r="L7" s="46" t="inlineStr">
+      <c r="K7" s="49" t="str"/>
+      <c r="L7" s="46" t="n"/>
+      <c r="M7" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2194,27 +2209,28 @@
       </c>
       <c r="B8" s="47" t="n"/>
       <c r="C8" s="47" t="n"/>
-      <c r="D8" s="46" t="inlineStr">
+      <c r="D8" s="47" t="n"/>
+      <c r="E8" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E8" s="47" t="n"/>
-      <c r="F8" s="46" t="inlineStr">
+      <c r="F8" s="47" t="n"/>
+      <c r="G8" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G8" s="48" t="n"/>
-      <c r="H8" s="47" t="n"/>
-      <c r="I8" s="46" t="inlineStr">
+      <c r="H8" s="48" t="n"/>
+      <c r="I8" s="47" t="n"/>
+      <c r="J8" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J8" s="49" t="str"/>
-      <c r="K8" s="46" t="n"/>
-      <c r="L8" s="46" t="inlineStr">
+      <c r="K8" s="49" t="str"/>
+      <c r="L8" s="46" t="n"/>
+      <c r="M8" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2228,27 +2244,28 @@
       </c>
       <c r="B9" s="47" t="n"/>
       <c r="C9" s="47" t="n"/>
-      <c r="D9" s="46" t="inlineStr">
+      <c r="D9" s="47" t="n"/>
+      <c r="E9" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E9" s="47" t="n"/>
-      <c r="F9" s="46" t="inlineStr">
+      <c r="F9" s="47" t="n"/>
+      <c r="G9" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G9" s="48" t="n"/>
-      <c r="H9" s="47" t="n"/>
-      <c r="I9" s="46" t="inlineStr">
+      <c r="H9" s="48" t="n"/>
+      <c r="I9" s="47" t="n"/>
+      <c r="J9" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J9" s="49" t="str"/>
-      <c r="K9" s="46" t="n"/>
-      <c r="L9" s="46" t="inlineStr">
+      <c r="K9" s="49" t="str"/>
+      <c r="L9" s="46" t="n"/>
+      <c r="M9" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2262,27 +2279,28 @@
       </c>
       <c r="B10" s="47" t="n"/>
       <c r="C10" s="47" t="n"/>
-      <c r="D10" s="46" t="inlineStr">
+      <c r="D10" s="47" t="n"/>
+      <c r="E10" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E10" s="47" t="n"/>
-      <c r="F10" s="46" t="inlineStr">
+      <c r="F10" s="47" t="n"/>
+      <c r="G10" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G10" s="48" t="n"/>
-      <c r="H10" s="47" t="n"/>
-      <c r="I10" s="46" t="inlineStr">
+      <c r="H10" s="48" t="n"/>
+      <c r="I10" s="47" t="n"/>
+      <c r="J10" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J10" s="49" t="str"/>
-      <c r="K10" s="46" t="n"/>
-      <c r="L10" s="46" t="inlineStr">
+      <c r="K10" s="49" t="str"/>
+      <c r="L10" s="46" t="n"/>
+      <c r="M10" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2296,27 +2314,28 @@
       </c>
       <c r="B11" s="47" t="n"/>
       <c r="C11" s="47" t="n"/>
-      <c r="D11" s="46" t="inlineStr">
+      <c r="D11" s="47" t="n"/>
+      <c r="E11" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E11" s="47" t="n"/>
-      <c r="F11" s="46" t="inlineStr">
+      <c r="F11" s="47" t="n"/>
+      <c r="G11" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G11" s="48" t="n"/>
-      <c r="H11" s="47" t="n"/>
-      <c r="I11" s="46" t="inlineStr">
+      <c r="H11" s="48" t="n"/>
+      <c r="I11" s="47" t="n"/>
+      <c r="J11" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J11" s="49" t="str"/>
-      <c r="K11" s="46" t="n"/>
-      <c r="L11" s="46" t="inlineStr">
+      <c r="K11" s="49" t="str"/>
+      <c r="L11" s="46" t="n"/>
+      <c r="M11" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2330,27 +2349,28 @@
       </c>
       <c r="B12" s="47" t="n"/>
       <c r="C12" s="47" t="n"/>
-      <c r="D12" s="46" t="inlineStr">
+      <c r="D12" s="47" t="n"/>
+      <c r="E12" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E12" s="47" t="n"/>
-      <c r="F12" s="46" t="inlineStr">
+      <c r="F12" s="47" t="n"/>
+      <c r="G12" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G12" s="48" t="n"/>
-      <c r="H12" s="47" t="n"/>
-      <c r="I12" s="46" t="inlineStr">
+      <c r="H12" s="48" t="n"/>
+      <c r="I12" s="47" t="n"/>
+      <c r="J12" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J12" s="49" t="str"/>
-      <c r="K12" s="46" t="n"/>
-      <c r="L12" s="46" t="inlineStr">
+      <c r="K12" s="49" t="str"/>
+      <c r="L12" s="46" t="n"/>
+      <c r="M12" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2364,27 +2384,28 @@
       </c>
       <c r="B13" s="47" t="n"/>
       <c r="C13" s="47" t="n"/>
-      <c r="D13" s="46" t="inlineStr">
+      <c r="D13" s="47" t="n"/>
+      <c r="E13" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E13" s="47" t="n"/>
-      <c r="F13" s="46" t="inlineStr">
+      <c r="F13" s="47" t="n"/>
+      <c r="G13" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G13" s="48" t="n"/>
-      <c r="H13" s="47" t="n"/>
-      <c r="I13" s="46" t="inlineStr">
+      <c r="H13" s="48" t="n"/>
+      <c r="I13" s="47" t="n"/>
+      <c r="J13" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J13" s="49" t="str"/>
-      <c r="K13" s="46" t="n"/>
-      <c r="L13" s="46" t="inlineStr">
+      <c r="K13" s="49" t="str"/>
+      <c r="L13" s="46" t="n"/>
+      <c r="M13" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2398,27 +2419,28 @@
       </c>
       <c r="B14" s="47" t="n"/>
       <c r="C14" s="47" t="n"/>
-      <c r="D14" s="46" t="inlineStr">
+      <c r="D14" s="47" t="n"/>
+      <c r="E14" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E14" s="47" t="n"/>
-      <c r="F14" s="46" t="inlineStr">
+      <c r="F14" s="47" t="n"/>
+      <c r="G14" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G14" s="48" t="n"/>
-      <c r="H14" s="47" t="n"/>
-      <c r="I14" s="46" t="inlineStr">
+      <c r="H14" s="48" t="n"/>
+      <c r="I14" s="47" t="n"/>
+      <c r="J14" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J14" s="49" t="str"/>
-      <c r="K14" s="46" t="n"/>
-      <c r="L14" s="46" t="inlineStr">
+      <c r="K14" s="49" t="str"/>
+      <c r="L14" s="46" t="n"/>
+      <c r="M14" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2432,27 +2454,28 @@
       </c>
       <c r="B15" s="47" t="n"/>
       <c r="C15" s="47" t="n"/>
-      <c r="D15" s="46" t="inlineStr">
+      <c r="D15" s="47" t="n"/>
+      <c r="E15" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E15" s="47" t="n"/>
-      <c r="F15" s="46" t="inlineStr">
+      <c r="F15" s="47" t="n"/>
+      <c r="G15" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G15" s="48" t="n"/>
-      <c r="H15" s="47" t="n"/>
-      <c r="I15" s="46" t="inlineStr">
+      <c r="H15" s="48" t="n"/>
+      <c r="I15" s="47" t="n"/>
+      <c r="J15" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J15" s="49" t="str"/>
-      <c r="K15" s="46" t="n"/>
-      <c r="L15" s="46" t="inlineStr">
+      <c r="K15" s="49" t="str"/>
+      <c r="L15" s="46" t="n"/>
+      <c r="M15" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2466,27 +2489,28 @@
       </c>
       <c r="B16" s="47" t="n"/>
       <c r="C16" s="47" t="n"/>
-      <c r="D16" s="46" t="inlineStr">
+      <c r="D16" s="47" t="n"/>
+      <c r="E16" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E16" s="47" t="n"/>
-      <c r="F16" s="46" t="inlineStr">
+      <c r="F16" s="47" t="n"/>
+      <c r="G16" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G16" s="48" t="n"/>
-      <c r="H16" s="47" t="n"/>
-      <c r="I16" s="46" t="inlineStr">
+      <c r="H16" s="48" t="n"/>
+      <c r="I16" s="47" t="n"/>
+      <c r="J16" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J16" s="49" t="str"/>
-      <c r="K16" s="46" t="n"/>
-      <c r="L16" s="46" t="inlineStr">
+      <c r="K16" s="49" t="str"/>
+      <c r="L16" s="46" t="n"/>
+      <c r="M16" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2500,27 +2524,28 @@
       </c>
       <c r="B17" s="47" t="n"/>
       <c r="C17" s="47" t="n"/>
-      <c r="D17" s="46" t="inlineStr">
+      <c r="D17" s="47" t="n"/>
+      <c r="E17" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E17" s="47" t="n"/>
-      <c r="F17" s="46" t="inlineStr">
+      <c r="F17" s="47" t="n"/>
+      <c r="G17" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G17" s="48" t="n"/>
-      <c r="H17" s="47" t="n"/>
-      <c r="I17" s="46" t="inlineStr">
+      <c r="H17" s="48" t="n"/>
+      <c r="I17" s="47" t="n"/>
+      <c r="J17" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J17" s="49" t="str"/>
-      <c r="K17" s="46" t="n"/>
-      <c r="L17" s="46" t="inlineStr">
+      <c r="K17" s="49" t="str"/>
+      <c r="L17" s="46" t="n"/>
+      <c r="M17" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2534,27 +2559,28 @@
       </c>
       <c r="B18" s="47" t="n"/>
       <c r="C18" s="47" t="n"/>
-      <c r="D18" s="46" t="inlineStr">
+      <c r="D18" s="47" t="n"/>
+      <c r="E18" s="46" t="inlineStr">
         <is>
           <t>计算值</t>
         </is>
       </c>
-      <c r="E18" s="47" t="n"/>
-      <c r="F18" s="46" t="inlineStr">
+      <c r="F18" s="47" t="n"/>
+      <c r="G18" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="G18" s="48" t="n"/>
-      <c r="H18" s="47" t="n"/>
-      <c r="I18" s="46" t="inlineStr">
+      <c r="H18" s="48" t="n"/>
+      <c r="I18" s="47" t="n"/>
+      <c r="J18" s="46" t="inlineStr">
         <is>
           <t>缺省值</t>
         </is>
       </c>
-      <c r="J18" s="49" t="str"/>
-      <c r="K18" s="46" t="n"/>
-      <c r="L18" s="46" t="inlineStr">
+      <c r="K18" s="49" t="str"/>
+      <c r="L18" s="46" t="n"/>
+      <c r="M18" s="46" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
@@ -2577,12 +2603,13 @@
       <c r="I19" s="45" t="n"/>
       <c r="J19" s="45" t="n"/>
       <c r="K19" s="45" t="n"/>
-      <c r="L19" s="43" t="n"/>
+      <c r="L19" s="45" t="n"/>
+      <c r="M19" s="43" t="n"/>
     </row>
     <row r="20" ht="27" customHeight="1" s="42">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>使用提示：目录参数由软件按核算期间解析，G列只读。自定义燃料在L列选“自定义”，所需单位热值含碳量填K列；填写值不自动视为实测。</t>
+          <t>使用提示：目录参数由软件按核算期间解析，H列只读。自定义燃料在M列选“自定义”，所需单位热值含碳量填L列；填写值不自动视为实测。消耗量须同时填写数据和单位。</t>
         </is>
       </c>
     </row>
@@ -2596,19 +2623,19 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="13">
-    <mergeCell ref="A20:L20"/>
-    <mergeCell ref="A21:L21"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="A20:M20"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="A2:A3"/>
     <mergeCell ref="K2:K3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="L2:L3"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:C18">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -2625,24 +2652,27 @@
       <formula>$I4="实测值"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="6">
-    <dataValidation sqref="C4:C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="当前不能填写" error="仅在相应数据来源选择“实测值”后可填写 C 列。" type="custom">
-      <formula1>OR($D4="实测值",C4="")</formula1>
+  <dataValidations count="7">
+    <dataValidation sqref="D4:D18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="当前不能填写" error="仅在相应数据来源选择“实测值”后可填写 C 列。" type="custom">
+      <formula1>OR($E4="实测值",D4="")</formula1>
     </dataValidation>
-    <dataValidation sqref="D4:D18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
+    <dataValidation sqref="E4:E18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
       <formula1>"计算值,实测值"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="当前不能填写" error="仅在相应数据来源选择“实测值”后可填写 E 列。" type="custom">
-      <formula1>OR($F4="实测值",$F4="填写值",E4="")</formula1>
+    <dataValidation sqref="F4:F18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="当前不能填写" error="仅在相应数据来源选择“实测值”后可填写 E 列。" type="custom">
+      <formula1>OR($G4="实测值",$G4="填写值",F4="")</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F18 I4:I18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
+    <dataValidation sqref="G4:G18 J4:J18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
       <formula1>"缺省值,实测值,填写值"</formula1>
     </dataValidation>
-    <dataValidation sqref="H4:H18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="当前不能填写" error="仅在相应数据来源选择“实测值”后可填写 H 列。" type="custom">
-      <formula1>OR($I4="实测值",$I4="填写值",H4="")</formula1>
+    <dataValidation sqref="I4:I18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="当前不能填写" error="仅在相应数据来源选择“实测值”后可填写 H 列。" type="custom">
+      <formula1>OR($J4="实测值",$J4="填写值",I4="")</formula1>
     </dataValidation>
-    <dataValidation sqref="L4:L18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="请核实填写值" error="请选择本列允许的选项。" type="list">
+    <dataValidation sqref="M4:M18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="请核实填写值" error="请选择本列允许的选项。" type="list">
       <formula1>"目录,自定义"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="请核实填写值" error="请选择本列允许的选项。" type="list">
+      <formula1>"t,10⁴Nm³"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor(input): preserve explicit process identities and shared electricity candidates
</commit_message>
<xml_diff>
--- a/resources/excel_templates/gb_t_32151_34_2024_appendix_b_v2.xlsx
+++ b/resources/excel_templates/gb_t_32151_34_2024_appendix_b_v2.xlsx
@@ -439,7 +439,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -858,6 +858,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF231F20"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1006,7 +1015,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1155,20 +1164,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="38" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
@@ -2685,14 +2689,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="29" customWidth="1" style="42" min="1" max="1"/>
-    <col width="27" customWidth="1" style="42" min="2" max="2"/>
+    <col width="25" customWidth="1" style="42" min="2" max="2"/>
+    <col width="26" customWidth="1" style="42" min="3" max="3"/>
     <col width="19" customWidth="1" style="42" min="3" max="3"/>
     <col width="23" customWidth="1" style="42" min="4" max="4"/>
     <col width="24" customWidth="1" style="42" min="5" max="5"/>
+    <col width="18" customWidth="1" style="42" min="7" max="7"/>
+    <col width="16" customWidth="1" style="42" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="42">
@@ -2702,41 +2709,67 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18.45" customHeight="1" s="42">
+    <row r="2" ht="26" customHeight="1" s="42">
       <c r="A2" s="16" t="inlineStr">
         <is>
           <t>物料名称ᵃ</t>
         </is>
       </c>
-      <c r="B2" s="51" t="n"/>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="B2" s="45" t="n"/>
+      <c r="C2" s="43" t="n"/>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>活动数据
 t</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>碳/挥发分含量</t>
         </is>
       </c>
-      <c r="E2" s="43" t="n"/>
-    </row>
-    <row r="3" ht="36.1" customHeight="1" s="42">
-      <c r="A3" s="52" t="n"/>
-      <c r="B3" s="53" t="n"/>
-      <c r="C3" s="44" t="n"/>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="F2" s="43" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>工序名称</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>物料序号</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1" s="42">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>分组</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>业务类别</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>实际名称</t>
+        </is>
+      </c>
+      <c r="D3" s="44" t="n"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>数值
 %</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
       </c>
+      <c r="G3" s="44" t="n"/>
+      <c r="H3" s="44" t="n"/>
     </row>
     <row r="4" ht="27.05" customHeight="1" s="42">
       <c r="A4" s="3" t="inlineStr">
@@ -2749,11 +2782,26 @@
           <t>待煅烧原料</t>
         </is>
       </c>
-      <c r="C4" s="47" t="n"/>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>待煅烧原料</t>
+        </is>
+      </c>
       <c r="D4" s="47" t="n"/>
-      <c r="E4" s="46" t="inlineStr">
+      <c r="E4" s="47" t="n"/>
+      <c r="F4" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>煅烧1</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>物料1</t>
         </is>
       </c>
     </row>
@@ -2768,11 +2816,26 @@
           <t>待煅烧原料</t>
         </is>
       </c>
-      <c r="C5" s="47" t="n"/>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>待煅烧原料</t>
+        </is>
+      </c>
       <c r="D5" s="47" t="n"/>
-      <c r="E5" s="46" t="inlineStr">
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>煅烧1</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
+        <is>
+          <t>物料1</t>
         </is>
       </c>
     </row>
@@ -2787,26 +2850,56 @@
           <t>煅后料</t>
         </is>
       </c>
-      <c r="C6" s="47" t="n"/>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>煅后料</t>
+        </is>
+      </c>
       <c r="D6" s="47" t="n"/>
-      <c r="E6" s="46" t="inlineStr">
+      <c r="E6" s="47" t="n"/>
+      <c r="F6" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
         </is>
       </c>
+      <c r="G6" s="46" t="inlineStr">
+        <is>
+          <t>煅烧1</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="inlineStr">
+        <is>
+          <t>物料2</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="27.05" customHeight="1" s="42">
-      <c r="A7" s="54" t="n"/>
+      <c r="A7" s="51" t="n"/>
       <c r="B7" s="46" t="inlineStr">
         <is>
           <t>欠烧煅料</t>
         </is>
       </c>
-      <c r="C7" s="47" t="n"/>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>欠烧煅料</t>
+        </is>
+      </c>
       <c r="D7" s="47" t="n"/>
-      <c r="E7" s="46" t="inlineStr">
+      <c r="E7" s="47" t="n"/>
+      <c r="F7" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>煅烧1</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="inlineStr">
+        <is>
+          <t>物料3</t>
         </is>
       </c>
     </row>
@@ -2817,11 +2910,26 @@
           <t>炭粉尘</t>
         </is>
       </c>
-      <c r="C8" s="47" t="n"/>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>炭粉尘</t>
+        </is>
+      </c>
       <c r="D8" s="47" t="n"/>
-      <c r="E8" s="46" t="inlineStr">
+      <c r="E8" s="47" t="n"/>
+      <c r="F8" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>煅烧1</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="inlineStr">
+        <is>
+          <t>物料4</t>
         </is>
       </c>
     </row>
@@ -2836,11 +2944,26 @@
           <t>煅后料</t>
         </is>
       </c>
-      <c r="C9" s="47" t="n"/>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>煅后料</t>
+        </is>
+      </c>
       <c r="D9" s="47" t="n"/>
-      <c r="E9" s="46" t="inlineStr">
+      <c r="E9" s="47" t="n"/>
+      <c r="F9" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>煅烧1</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="inlineStr">
+        <is>
+          <t>物料2</t>
         </is>
       </c>
     </row>
@@ -2851,9 +2974,9 @@
         </is>
       </c>
       <c r="B10" s="43" t="n"/>
-      <c r="C10" s="55" t="n"/>
-      <c r="D10" s="45" t="n"/>
-      <c r="E10" s="43" t="n"/>
+      <c r="D10" s="52" t="n"/>
+      <c r="E10" s="45" t="n"/>
+      <c r="F10" s="43" t="n"/>
     </row>
     <row r="11" ht="18.45" customHeight="1" s="42">
       <c r="A11" s="35" t="inlineStr">
@@ -2864,7 +2987,10 @@
       <c r="B11" s="45" t="n"/>
       <c r="C11" s="45" t="n"/>
       <c r="D11" s="45" t="n"/>
-      <c r="E11" s="43" t="n"/>
+      <c r="E11" s="45" t="n"/>
+      <c r="F11" s="45" t="n"/>
+      <c r="G11" s="45" t="n"/>
+      <c r="H11" s="43" t="n"/>
     </row>
     <row r="12" ht="27" customHeight="1" s="42">
       <c r="A12" s="15" t="inlineStr">
@@ -2873,29 +2999,31 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="27" customHeight="1" s="42">
+    <row r="13" ht="36" customHeight="1" s="42">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>数据来源：目前仅允许选择“实测值”；化学计算、缺省值（暂不可选择）。</t>
+          <t>填写提示：同一工序、同一物料的碳与挥发分行使用相同物料序号、名称和活动数据；新增物料给出独立序号，新增工序给出独立名称。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="10">
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A2:B3"/>
-    <mergeCell ref="D2:E2"/>
+  <mergeCells count="12">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D10:F10"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E4:E9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
+    <dataValidation sqref="F4:F9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
       <formula1>"实测值"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2909,14 +3037,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="29" customWidth="1" style="42" min="1" max="1"/>
-    <col width="27" customWidth="1" style="42" min="2" max="2"/>
+    <col width="25" customWidth="1" style="42" min="2" max="2"/>
+    <col width="26" customWidth="1" style="42" min="3" max="3"/>
     <col width="19" customWidth="1" style="42" min="3" max="3"/>
     <col width="23" customWidth="1" style="42" min="4" max="4"/>
     <col width="24" customWidth="1" style="42" min="5" max="5"/>
+    <col width="18" customWidth="1" style="42" min="7" max="7"/>
+    <col width="16" customWidth="1" style="42" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="42">
@@ -2926,41 +3057,67 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18.45" customHeight="1" s="42">
+    <row r="2" ht="26" customHeight="1" s="42">
       <c r="A2" s="30" t="inlineStr">
         <is>
           <t>物料名称ᵃ</t>
         </is>
       </c>
-      <c r="B2" s="56" t="n"/>
-      <c r="C2" s="32" t="inlineStr">
+      <c r="B2" s="53" t="n"/>
+      <c r="C2" s="54" t="n"/>
+      <c r="D2" s="32" t="inlineStr">
         <is>
           <t>活动数据
 t</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="E2" s="32" t="inlineStr">
         <is>
           <t>碳/挥发分含量</t>
         </is>
       </c>
-      <c r="E2" s="57" t="n"/>
-    </row>
-    <row r="3" ht="36.1" customHeight="1" s="42">
-      <c r="A3" s="58" t="n"/>
-      <c r="B3" s="57" t="n"/>
-      <c r="C3" s="59" t="n"/>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="F2" s="54" t="n"/>
+      <c r="G2" s="32" t="inlineStr">
+        <is>
+          <t>工序名称</t>
+        </is>
+      </c>
+      <c r="H2" s="32" t="inlineStr">
+        <is>
+          <t>物料序号</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1" s="42">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>分组</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>业务类别</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>实际名称</t>
+        </is>
+      </c>
+      <c r="D3" s="55" t="n"/>
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>数值
 %</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
       </c>
+      <c r="G3" s="55" t="n"/>
+      <c r="H3" s="55" t="n"/>
     </row>
     <row r="4" ht="18.05" customHeight="1" s="42">
       <c r="A4" s="18" t="inlineStr">
@@ -2974,26 +3131,56 @@
           <t>填充料</t>
         </is>
       </c>
-      <c r="C4" s="47" t="n"/>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>填充料</t>
+        </is>
+      </c>
       <c r="D4" s="47" t="n"/>
-      <c r="E4" s="46" t="inlineStr">
+      <c r="E4" s="47" t="n"/>
+      <c r="F4" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
         </is>
       </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>焙烧1</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>物料1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18.05" customHeight="1" s="42">
-      <c r="A5" s="59" t="n"/>
+      <c r="A5" s="55" t="n"/>
       <c r="B5" s="46" t="inlineStr">
         <is>
           <t>待焙烧(炭化)品</t>
         </is>
       </c>
-      <c r="C5" s="47" t="n"/>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>待焙烧(炭化)品</t>
+        </is>
+      </c>
       <c r="D5" s="47" t="n"/>
-      <c r="E5" s="46" t="inlineStr">
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>焙烧1</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
+        <is>
+          <t>物料2</t>
         </is>
       </c>
     </row>
@@ -3009,26 +3196,56 @@
           <t>填充料</t>
         </is>
       </c>
-      <c r="C6" s="47" t="n"/>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>填充料</t>
+        </is>
+      </c>
       <c r="D6" s="47" t="n"/>
-      <c r="E6" s="46" t="inlineStr">
+      <c r="E6" s="47" t="n"/>
+      <c r="F6" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
         </is>
       </c>
+      <c r="G6" s="46" t="inlineStr">
+        <is>
+          <t>焙烧1</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="inlineStr">
+        <is>
+          <t>物料1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18.05" customHeight="1" s="42">
-      <c r="A7" s="59" t="n"/>
+      <c r="A7" s="55" t="n"/>
       <c r="B7" s="46" t="inlineStr">
         <is>
           <t>待焙烧(炭化)品</t>
         </is>
       </c>
-      <c r="C7" s="47" t="n"/>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>待焙烧(炭化)品</t>
+        </is>
+      </c>
       <c r="D7" s="47" t="n"/>
-      <c r="E7" s="46" t="inlineStr">
+      <c r="E7" s="47" t="n"/>
+      <c r="F7" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>焙烧1</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="inlineStr">
+        <is>
+          <t>物料2</t>
         </is>
       </c>
     </row>
@@ -3044,26 +3261,56 @@
           <t>粉尘 、碎屑 、副产品等</t>
         </is>
       </c>
-      <c r="C8" s="47" t="n"/>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>粉尘 、碎屑 、副产品等</t>
+        </is>
+      </c>
       <c r="D8" s="47" t="n"/>
-      <c r="E8" s="46" t="inlineStr">
+      <c r="E8" s="47" t="n"/>
+      <c r="F8" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
         </is>
       </c>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>焙烧1</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="inlineStr">
+        <is>
+          <t>物料3</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18.05" customHeight="1" s="42">
-      <c r="A9" s="59" t="n"/>
+      <c r="A9" s="55" t="n"/>
       <c r="B9" s="46" t="inlineStr">
         <is>
           <t>焙烧(炭化)品</t>
         </is>
       </c>
-      <c r="C9" s="47" t="n"/>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>焙烧(炭化)品</t>
+        </is>
+      </c>
       <c r="D9" s="47" t="n"/>
-      <c r="E9" s="46" t="inlineStr">
+      <c r="E9" s="47" t="n"/>
+      <c r="F9" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>焙烧1</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="inlineStr">
+        <is>
+          <t>物料4</t>
         </is>
       </c>
     </row>
@@ -3074,9 +3321,9 @@
         </is>
       </c>
       <c r="B10" s="43" t="n"/>
-      <c r="C10" s="55" t="n"/>
-      <c r="D10" s="45" t="n"/>
-      <c r="E10" s="43" t="n"/>
+      <c r="D10" s="52" t="n"/>
+      <c r="E10" s="45" t="n"/>
+      <c r="F10" s="43" t="n"/>
     </row>
     <row r="11" ht="18.45" customHeight="1" s="42">
       <c r="A11" s="29" t="inlineStr">
@@ -3084,10 +3331,13 @@
           <t xml:space="preserve">       a     报告主体根据实际投入产出情况 ,可自行加行一一列明并填数 。</t>
         </is>
       </c>
-      <c r="B11" s="60" t="n"/>
-      <c r="C11" s="60" t="n"/>
-      <c r="D11" s="60" t="n"/>
-      <c r="E11" s="61" t="n"/>
+      <c r="B11" s="56" t="n"/>
+      <c r="C11" s="56" t="n"/>
+      <c r="D11" s="56" t="n"/>
+      <c r="E11" s="56" t="n"/>
+      <c r="F11" s="56" t="n"/>
+      <c r="G11" s="56" t="n"/>
+      <c r="H11" s="57" t="n"/>
     </row>
     <row r="12" ht="27" customHeight="1" s="42">
       <c r="A12" s="15" t="inlineStr">
@@ -3096,31 +3346,33 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="27" customHeight="1" s="42">
+    <row r="13" ht="36" customHeight="1" s="42">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>数据来源：目前仅允许选择“实测值”；化学计算、缺省值（暂不可选择）。</t>
+          <t>填写提示：同一工序、同一物料的碳与挥发分行使用相同物料序号、名称和活动数据；新增物料给出独立序号，新增工序给出独立名称。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="12">
-    <mergeCell ref="A12:E12"/>
+  <mergeCells count="14">
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A2:B3"/>
-    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="E2:F2"/>
     <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D10:F10"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E4:E9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
+    <dataValidation sqref="F4:F9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
       <formula1>"实测值"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3134,14 +3386,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="29" customWidth="1" style="42" min="1" max="1"/>
-    <col width="27" customWidth="1" style="42" min="2" max="2"/>
+    <col width="25" customWidth="1" style="42" min="2" max="2"/>
+    <col width="26" customWidth="1" style="42" min="3" max="3"/>
     <col width="19" customWidth="1" style="42" min="3" max="3"/>
     <col width="23" customWidth="1" style="42" min="4" max="4"/>
     <col width="24" customWidth="1" style="42" min="5" max="5"/>
+    <col width="18" customWidth="1" style="42" min="7" max="7"/>
+    <col width="16" customWidth="1" style="42" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="42">
@@ -3151,41 +3406,67 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="42">
+    <row r="2" ht="26" customHeight="1" s="42">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>物料名称ᵃ</t>
         </is>
       </c>
-      <c r="B2" s="62" t="n"/>
-      <c r="C2" s="19" t="inlineStr">
+      <c r="B2" s="56" t="n"/>
+      <c r="C2" s="57" t="n"/>
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>活动数据
 t</t>
         </is>
       </c>
-      <c r="D2" s="19" t="inlineStr">
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>碳/挥发分含量</t>
         </is>
       </c>
-      <c r="E2" s="61" t="n"/>
-    </row>
-    <row r="3" ht="33" customHeight="1" s="42">
-      <c r="A3" s="58" t="n"/>
-      <c r="B3" s="57" t="n"/>
-      <c r="C3" s="59" t="n"/>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="F2" s="57" t="n"/>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>工序名称</t>
+        </is>
+      </c>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>物料序号</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1" s="42">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>分组</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>业务类别</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>实际名称</t>
+        </is>
+      </c>
+      <c r="D3" s="55" t="n"/>
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>数值
 %</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
       </c>
+      <c r="G3" s="55" t="n"/>
+      <c r="H3" s="55" t="n"/>
     </row>
     <row r="4" ht="16.5" customHeight="1" s="42">
       <c r="A4" s="19" t="inlineStr">
@@ -3199,26 +3480,56 @@
           <t>保温料和电阻料</t>
         </is>
       </c>
-      <c r="C4" s="47" t="n"/>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>保温料和电阻料</t>
+        </is>
+      </c>
       <c r="D4" s="47" t="n"/>
-      <c r="E4" s="46" t="inlineStr">
+      <c r="E4" s="47" t="n"/>
+      <c r="F4" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
         </is>
       </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>石墨化1</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>物料1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="42">
-      <c r="A5" s="59" t="n"/>
+      <c r="A5" s="55" t="n"/>
       <c r="B5" s="46" t="inlineStr">
         <is>
           <t>待石墨化品</t>
         </is>
       </c>
-      <c r="C5" s="47" t="n"/>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>待石墨化品</t>
+        </is>
+      </c>
       <c r="D5" s="47" t="n"/>
-      <c r="E5" s="46" t="inlineStr">
+      <c r="E5" s="47" t="n"/>
+      <c r="F5" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>石墨化1</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
+        <is>
+          <t>物料2</t>
         </is>
       </c>
     </row>
@@ -3234,11 +3545,26 @@
           <t>保温料和电阻料</t>
         </is>
       </c>
-      <c r="C6" s="47" t="n"/>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>保温料和电阻料</t>
+        </is>
+      </c>
       <c r="D6" s="47" t="n"/>
-      <c r="E6" s="46" t="inlineStr">
+      <c r="E6" s="47" t="n"/>
+      <c r="F6" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G6" s="46" t="inlineStr">
+        <is>
+          <t>石墨化1</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="inlineStr">
+        <is>
+          <t>物料1</t>
         </is>
       </c>
     </row>
@@ -3255,26 +3581,57 @@
 副产品等</t>
         </is>
       </c>
-      <c r="C7" s="47" t="n"/>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>粉尘 、碎屑 、残块(渣) 、
+副产品等</t>
+        </is>
+      </c>
       <c r="D7" s="47" t="n"/>
-      <c r="E7" s="46" t="inlineStr">
+      <c r="E7" s="47" t="n"/>
+      <c r="F7" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
         </is>
       </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>石墨化1</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="inlineStr">
+        <is>
+          <t>物料3</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="16.5" customHeight="1" s="42">
-      <c r="A8" s="59" t="n"/>
+      <c r="A8" s="55" t="n"/>
       <c r="B8" s="46" t="inlineStr">
         <is>
           <t>石墨化产品</t>
         </is>
       </c>
-      <c r="C8" s="47" t="n"/>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>石墨化产品</t>
+        </is>
+      </c>
       <c r="D8" s="47" t="n"/>
-      <c r="E8" s="46" t="inlineStr">
+      <c r="E8" s="47" t="n"/>
+      <c r="F8" s="46" t="inlineStr">
         <is>
           <t>实测值</t>
+        </is>
+      </c>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>石墨化1</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="inlineStr">
+        <is>
+          <t>物料4</t>
         </is>
       </c>
     </row>
@@ -3285,9 +3642,9 @@
         </is>
       </c>
       <c r="B9" s="43" t="n"/>
-      <c r="C9" s="55" t="n"/>
-      <c r="D9" s="45" t="n"/>
-      <c r="E9" s="43" t="n"/>
+      <c r="D9" s="52" t="n"/>
+      <c r="E9" s="45" t="n"/>
+      <c r="F9" s="43" t="n"/>
     </row>
     <row r="10" ht="16.5" customHeight="1" s="42">
       <c r="A10" s="29" t="inlineStr">
@@ -3295,10 +3652,13 @@
           <t xml:space="preserve">       a     报告主体根据实际投入产出情况 ,可自行加行一一列明并填数 。</t>
         </is>
       </c>
-      <c r="B10" s="60" t="n"/>
-      <c r="C10" s="60" t="n"/>
-      <c r="D10" s="60" t="n"/>
-      <c r="E10" s="61" t="n"/>
+      <c r="B10" s="56" t="n"/>
+      <c r="C10" s="56" t="n"/>
+      <c r="D10" s="56" t="n"/>
+      <c r="E10" s="56" t="n"/>
+      <c r="F10" s="56" t="n"/>
+      <c r="G10" s="56" t="n"/>
+      <c r="H10" s="57" t="n"/>
     </row>
     <row r="11" ht="27" customHeight="1" s="42">
       <c r="A11" s="15" t="inlineStr">
@@ -3307,30 +3667,32 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="27" customHeight="1" s="42">
+    <row r="12" ht="36" customHeight="1" s="42">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>数据来源：目前仅允许选择“实测值”；化学计算、缺省值（暂不可选择）。</t>
+          <t>填写提示：同一工序、同一物料的碳与挥发分行使用相同物料序号、名称和活动数据；新增物料给出独立序号，新增工序给出独立名称。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="11">
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A2:B3"/>
-    <mergeCell ref="D2:E2"/>
+  <mergeCells count="13">
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="D9:F9"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E4:E8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
+    <dataValidation sqref="F4:F8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="请选择有效选项" error="此字段只能从下拉列表中选择。" type="list">
       <formula1>"实测值"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3553,8 +3915,8 @@
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" s="42">
-      <c r="A3" s="63" t="n"/>
-      <c r="B3" s="63" t="n"/>
+      <c r="A3" s="58" t="n"/>
+      <c r="B3" s="58" t="n"/>
       <c r="C3" s="50" t="inlineStr">
         <is>
           <t>CaCO₃</t>
@@ -3572,8 +3934,8 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" s="42">
-      <c r="A4" s="64" t="n"/>
-      <c r="B4" s="64" t="n"/>
+      <c r="A4" s="59" t="n"/>
+      <c r="B4" s="59" t="n"/>
       <c r="C4" s="50" t="inlineStr">
         <is>
           <t>MgCO₃</t>
@@ -3591,8 +3953,8 @@
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" s="42">
-      <c r="A5" s="59" t="n"/>
-      <c r="B5" s="59" t="n"/>
+      <c r="A5" s="55" t="n"/>
+      <c r="B5" s="55" t="n"/>
       <c r="C5" s="50" t="inlineStr">
         <is>
           <t>其他</t>
@@ -3610,8 +3972,8 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" s="42">
-      <c r="A6" s="63" t="n"/>
-      <c r="B6" s="63" t="n"/>
+      <c r="A6" s="58" t="n"/>
+      <c r="B6" s="58" t="n"/>
       <c r="C6" s="50" t="n"/>
       <c r="D6" s="47" t="n"/>
       <c r="E6" s="7" t="n"/>
@@ -3625,8 +3987,8 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" s="42">
-      <c r="A7" s="64" t="n"/>
-      <c r="B7" s="64" t="n"/>
+      <c r="A7" s="59" t="n"/>
+      <c r="B7" s="59" t="n"/>
       <c r="C7" s="50" t="n"/>
       <c r="D7" s="47" t="n"/>
       <c r="E7" s="7" t="n"/>
@@ -3640,8 +4002,8 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" s="42">
-      <c r="A8" s="59" t="n"/>
-      <c r="B8" s="59" t="n"/>
+      <c r="A8" s="55" t="n"/>
+      <c r="B8" s="55" t="n"/>
       <c r="C8" s="50" t="n"/>
       <c r="D8" s="47" t="n"/>
       <c r="E8" s="7" t="n"/>
@@ -3668,7 +4030,7 @@
       <c r="F9" s="45" t="n"/>
       <c r="G9" s="45" t="n"/>
       <c r="H9" s="45" t="n"/>
-      <c r="I9" s="65" t="n"/>
+      <c r="I9" s="60" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -3750,7 +4112,7 @@
       </c>
       <c r="B3" s="47" t="n"/>
       <c r="C3" s="47" t="n"/>
-      <c r="D3" s="66" t="n"/>
+      <c r="D3" s="61" t="n"/>
       <c r="E3" s="49" t="str"/>
     </row>
     <row r="4" ht="16.5" customHeight="1" s="42">
@@ -3761,7 +4123,7 @@
       </c>
       <c r="B4" s="47" t="n"/>
       <c r="C4" s="47" t="n"/>
-      <c r="D4" s="66" t="n"/>
+      <c r="D4" s="61" t="n"/>
       <c r="E4" s="49" t="str"/>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="42">
@@ -3773,7 +4135,7 @@
       <c r="B5" s="45" t="n"/>
       <c r="C5" s="45" t="n"/>
       <c r="D5" s="45" t="n"/>
-      <c r="E5" s="65" t="n"/>
+      <c r="E5" s="60" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -3864,9 +4226,9 @@
       <c r="B3" s="47" t="n"/>
       <c r="C3" s="47" t="n"/>
       <c r="D3" s="47" t="n"/>
-      <c r="E3" s="66" t="n"/>
-      <c r="F3" s="66" t="n"/>
-      <c r="G3" s="67" t="n">
+      <c r="E3" s="61" t="n"/>
+      <c r="F3" s="61" t="n"/>
+      <c r="G3" s="62" t="n">
         <v>0.11</v>
       </c>
     </row>
@@ -3879,9 +4241,9 @@
       <c r="B4" s="47" t="n"/>
       <c r="C4" s="47" t="n"/>
       <c r="D4" s="47" t="n"/>
-      <c r="E4" s="66" t="n"/>
-      <c r="F4" s="66" t="n"/>
-      <c r="G4" s="67" t="n">
+      <c r="E4" s="61" t="n"/>
+      <c r="F4" s="61" t="n"/>
+      <c r="G4" s="62" t="n">
         <v>0.11</v>
       </c>
     </row>
@@ -3896,7 +4258,7 @@
       <c r="D5" s="45" t="n"/>
       <c r="E5" s="45" t="n"/>
       <c r="F5" s="45" t="n"/>
-      <c r="G5" s="65" t="n"/>
+      <c r="G5" s="60" t="n"/>
     </row>
     <row r="6" ht="27" customHeight="1" s="42">
       <c r="A6" s="15" t="inlineStr">

</xml_diff>